<commit_message>
6个语音。 无梦 QQ 1744500392
</commit_message>
<xml_diff>
--- a/Iocp20Coroutine/表/单位.xlsx
+++ b/Iocp20Coroutine/表/单位.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12255"/>
+    <workbookView windowWidth="28800" windowHeight="12255" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="单位" sheetId="3" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="718" uniqueCount="338">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="718" uniqueCount="339">
   <si>
     <t>类型</t>
   </si>
@@ -219,355 +219,358 @@
     <t>活动单位/工虫</t>
   </si>
   <si>
+    <t>语音/是男声年轻</t>
+  </si>
+  <si>
+    <t>待机</t>
+  </si>
+  <si>
+    <t>died</t>
+  </si>
+  <si>
+    <t>音效/zdrDth00</t>
+  </si>
+  <si>
+    <t>可采集资源，可变成建筑</t>
+  </si>
+  <si>
+    <t>飞机</t>
+  </si>
+  <si>
+    <t>活动单位/飞机</t>
+  </si>
+  <si>
+    <t>音效/飞机声</t>
+  </si>
+  <si>
+    <t>p_plane_01</t>
+  </si>
+  <si>
+    <t>flight_04</t>
+  </si>
+  <si>
+    <t>slide</t>
+  </si>
+  <si>
+    <t>可飞越障碍物</t>
+  </si>
+  <si>
+    <t>枪虫</t>
+  </si>
+  <si>
+    <t>活动单位/枪虫</t>
+  </si>
+  <si>
+    <t>音效/zhyWht01</t>
+  </si>
+  <si>
+    <t>m_78</t>
+  </si>
+  <si>
+    <t>音效/zhyDth00</t>
+  </si>
+  <si>
+    <t>近战虫</t>
+  </si>
+  <si>
+    <t>活动单位/近战虫</t>
+  </si>
+  <si>
+    <t>音效/ZZeWht00</t>
+  </si>
+  <si>
+    <t>chongmu_01</t>
+  </si>
+  <si>
+    <t>音效/ZZeDth00</t>
+  </si>
+  <si>
+    <t>幼虫</t>
+  </si>
+  <si>
+    <t>活动单位/幼虫</t>
+  </si>
+  <si>
+    <t>音效/ZLaWht00</t>
+  </si>
+  <si>
+    <t>幼虫已加动作</t>
+  </si>
+  <si>
+    <t>Armature|Armature.001|Take 001|BaseLayer</t>
+  </si>
+  <si>
+    <t>Armature|Armature.004|Take 001|BaseLayer</t>
+  </si>
+  <si>
+    <t>音效/ZLaDth00</t>
+  </si>
+  <si>
+    <t>可蜕变为其它活动单位</t>
+  </si>
+  <si>
+    <t>绿色坦克</t>
+  </si>
+  <si>
+    <t>活动单位/绿色坦克</t>
+  </si>
+  <si>
+    <t>音效/ZLaPss00</t>
+  </si>
+  <si>
+    <t>p_B_tank_01</t>
+  </si>
+  <si>
+    <t>超远距离发射光刺，光刺会遭到障碍物阻挡。</t>
+  </si>
+  <si>
+    <t>光刺</t>
+  </si>
+  <si>
+    <t>活动单位/光刺</t>
+  </si>
+  <si>
+    <t>房虫</t>
+  </si>
+  <si>
+    <t>活动单位/房虫</t>
+  </si>
+  <si>
+    <t>音效/zovWht00</t>
+  </si>
+  <si>
+    <t>骨架|stand</t>
+  </si>
+  <si>
+    <t>骨架|death</t>
+  </si>
+  <si>
+    <t>音效/zovDth00</t>
+  </si>
+  <si>
+    <t>可增加活动单位上限</t>
+  </si>
+  <si>
+    <t>飞虫</t>
+  </si>
+  <si>
+    <t>活动单位/飞虫</t>
+  </si>
+  <si>
+    <t>音效/zmuWht01</t>
+  </si>
+  <si>
+    <t>飞虫-动作</t>
+  </si>
+  <si>
+    <t>音效/zmuDth00</t>
+  </si>
+  <si>
+    <t>可飞跃障碍物</t>
+  </si>
+  <si>
+    <t>医疗兵</t>
+  </si>
+  <si>
+    <t>活动单位/医疗兵</t>
+  </si>
+  <si>
+    <t>语音/TMdWht00</t>
+  </si>
+  <si>
+    <t>Dwarf Idle</t>
+  </si>
+  <si>
+    <t>语音/TMdDth00</t>
+  </si>
+  <si>
+    <t>可给友方单位恢复HP</t>
+  </si>
+  <si>
+    <t>防空兵</t>
+  </si>
+  <si>
+    <t>活动单位/防空兵</t>
+  </si>
+  <si>
+    <t>p_C_rpg_02</t>
+  </si>
+  <si>
+    <t>远程对空范围攻击，爆炸溅射会伤害己方单位，不可对地攻击</t>
+  </si>
+  <si>
+    <t>基地</t>
+  </si>
+  <si>
+    <t>建筑/基地</t>
+  </si>
+  <si>
+    <t>p_Base_02</t>
+  </si>
+  <si>
+    <t>die</t>
+  </si>
+  <si>
+    <t>explo4</t>
+  </si>
+  <si>
+    <t>可产出工程车</t>
+  </si>
+  <si>
+    <t>兵营</t>
+  </si>
+  <si>
+    <t>建筑/兵营</t>
+  </si>
+  <si>
+    <t>Factory_leaye</t>
+  </si>
+  <si>
+    <t>兵营空闲</t>
+  </si>
+  <si>
+    <t>Take 001</t>
+  </si>
+  <si>
+    <t>EXPLOMED</t>
+  </si>
+  <si>
+    <t>可产出枪兵和近战兵</t>
+  </si>
+  <si>
+    <t>民房</t>
+  </si>
+  <si>
+    <t>建筑/民房</t>
+  </si>
+  <si>
+    <t>地堡</t>
+  </si>
+  <si>
+    <t>建筑/地堡</t>
+  </si>
+  <si>
+    <t>地堡872面</t>
+  </si>
+  <si>
+    <t>高HP，可派遣步兵进入地堡</t>
+  </si>
+  <si>
+    <t>炮台</t>
+  </si>
+  <si>
+    <t>建筑/炮台</t>
+  </si>
+  <si>
+    <t>p_jiqiangbao_d_01</t>
+  </si>
+  <si>
+    <t>show</t>
+  </si>
+  <si>
+    <t>音效/explo1</t>
+  </si>
+  <si>
+    <t>克制除了坦克以外的一切单位</t>
+  </si>
+  <si>
+    <t>虫巢</t>
+  </si>
+  <si>
+    <t>建筑/虫巢</t>
+  </si>
+  <si>
+    <t>音效/zhaWht00</t>
+  </si>
+  <si>
+    <t>hatchery_skin</t>
+  </si>
+  <si>
+    <t>音效/ZBldgDth</t>
+  </si>
+  <si>
+    <t>可产出幼虫</t>
+  </si>
+  <si>
+    <t>机场</t>
+  </si>
+  <si>
+    <t>建筑/机场</t>
+  </si>
+  <si>
+    <t>airport_500_1mesh</t>
+  </si>
+  <si>
+    <t>可产出飞机</t>
+  </si>
+  <si>
+    <t>重车厂</t>
+  </si>
+  <si>
+    <t>建筑/重车厂</t>
+  </si>
+  <si>
+    <t>风扇飞</t>
+  </si>
+  <si>
+    <t>重车厂Idle</t>
+  </si>
+  <si>
+    <t>可产出三色坦克</t>
+  </si>
+  <si>
+    <t>虫营</t>
+  </si>
+  <si>
+    <t>建筑/虫营</t>
+  </si>
+  <si>
+    <t>音效/zspWht00</t>
+  </si>
+  <si>
+    <t>近战虫和枪虫的前置建筑，只需1个就够了</t>
+  </si>
+  <si>
+    <t>飞塔</t>
+  </si>
+  <si>
+    <t>建筑/飞塔</t>
+  </si>
+  <si>
+    <t>音效/zscWht00</t>
+  </si>
+  <si>
+    <t>飞虫的前置建筑，只需1个就够了</t>
+  </si>
+  <si>
+    <t>拟态源</t>
+  </si>
+  <si>
+    <t>建筑/拟态源</t>
+  </si>
+  <si>
+    <t>绿色坦克的前置建筑，只需1个就够了</t>
+  </si>
+  <si>
+    <t>太岁</t>
+  </si>
+  <si>
+    <t>建筑/太岁</t>
+  </si>
+  <si>
+    <t>可扩张苔蔓(wàn)，扩张完成后可分裂另一个太岁</t>
+  </si>
+  <si>
+    <t>枪虫怪</t>
+  </si>
+  <si>
+    <t>近战虫怪</t>
+  </si>
+  <si>
+    <t>工怪</t>
+  </si>
+  <si>
     <t>音效/zdrWht00</t>
-  </si>
-  <si>
-    <t>待机</t>
-  </si>
-  <si>
-    <t>died</t>
-  </si>
-  <si>
-    <t>音效/zdrDth00</t>
-  </si>
-  <si>
-    <t>可采集资源，可变成建筑</t>
-  </si>
-  <si>
-    <t>飞机</t>
-  </si>
-  <si>
-    <t>活动单位/飞机</t>
-  </si>
-  <si>
-    <t>音效/飞机声</t>
-  </si>
-  <si>
-    <t>p_plane_01</t>
-  </si>
-  <si>
-    <t>flight_04</t>
-  </si>
-  <si>
-    <t>slide</t>
-  </si>
-  <si>
-    <t>可飞越障碍物</t>
-  </si>
-  <si>
-    <t>枪虫</t>
-  </si>
-  <si>
-    <t>活动单位/枪虫</t>
-  </si>
-  <si>
-    <t>音效/zhyWht01</t>
-  </si>
-  <si>
-    <t>m_78</t>
-  </si>
-  <si>
-    <t>音效/zhyDth00</t>
-  </si>
-  <si>
-    <t>近战虫</t>
-  </si>
-  <si>
-    <t>活动单位/近战虫</t>
-  </si>
-  <si>
-    <t>音效/ZZeWht00</t>
-  </si>
-  <si>
-    <t>chongmu_01</t>
-  </si>
-  <si>
-    <t>音效/ZZeDth00</t>
-  </si>
-  <si>
-    <t>幼虫</t>
-  </si>
-  <si>
-    <t>活动单位/幼虫</t>
-  </si>
-  <si>
-    <t>音效/ZLaWht00</t>
-  </si>
-  <si>
-    <t>幼虫已加动作</t>
-  </si>
-  <si>
-    <t>Armature|Armature.001|Take 001|BaseLayer</t>
-  </si>
-  <si>
-    <t>Armature|Armature.004|Take 001|BaseLayer</t>
-  </si>
-  <si>
-    <t>音效/ZLaDth00</t>
-  </si>
-  <si>
-    <t>可蜕变为其它活动单位</t>
-  </si>
-  <si>
-    <t>绿色坦克</t>
-  </si>
-  <si>
-    <t>活动单位/绿色坦克</t>
-  </si>
-  <si>
-    <t>音效/ZLaPss00</t>
-  </si>
-  <si>
-    <t>p_B_tank_01</t>
-  </si>
-  <si>
-    <t>超远距离发射光刺，光刺会遭到障碍物阻挡。</t>
-  </si>
-  <si>
-    <t>光刺</t>
-  </si>
-  <si>
-    <t>活动单位/光刺</t>
-  </si>
-  <si>
-    <t>房虫</t>
-  </si>
-  <si>
-    <t>活动单位/房虫</t>
-  </si>
-  <si>
-    <t>音效/zovWht00</t>
-  </si>
-  <si>
-    <t>骨架|stand</t>
-  </si>
-  <si>
-    <t>骨架|death</t>
-  </si>
-  <si>
-    <t>音效/zovDth00</t>
-  </si>
-  <si>
-    <t>可增加活动单位上限</t>
-  </si>
-  <si>
-    <t>飞虫</t>
-  </si>
-  <si>
-    <t>活动单位/飞虫</t>
-  </si>
-  <si>
-    <t>音效/zmuWht01</t>
-  </si>
-  <si>
-    <t>飞虫-动作</t>
-  </si>
-  <si>
-    <t>音效/zmuDth00</t>
-  </si>
-  <si>
-    <t>可飞跃障碍物</t>
-  </si>
-  <si>
-    <t>医疗兵</t>
-  </si>
-  <si>
-    <t>活动单位/医疗兵</t>
-  </si>
-  <si>
-    <t>语音/TMdWht00</t>
-  </si>
-  <si>
-    <t>Dwarf Idle</t>
-  </si>
-  <si>
-    <t>语音/TMdDth00</t>
-  </si>
-  <si>
-    <t>可给友方单位恢复HP</t>
-  </si>
-  <si>
-    <t>防空兵</t>
-  </si>
-  <si>
-    <t>活动单位/防空兵</t>
-  </si>
-  <si>
-    <t>p_C_rpg_02</t>
-  </si>
-  <si>
-    <t>远程对空范围攻击，爆炸溅射会伤害己方单位，不可对地攻击</t>
-  </si>
-  <si>
-    <t>基地</t>
-  </si>
-  <si>
-    <t>建筑/基地</t>
-  </si>
-  <si>
-    <t>p_Base_02</t>
-  </si>
-  <si>
-    <t>die</t>
-  </si>
-  <si>
-    <t>explo4</t>
-  </si>
-  <si>
-    <t>可产出工程车</t>
-  </si>
-  <si>
-    <t>兵营</t>
-  </si>
-  <si>
-    <t>建筑/兵营</t>
-  </si>
-  <si>
-    <t>Factory_leaye</t>
-  </si>
-  <si>
-    <t>兵营空闲</t>
-  </si>
-  <si>
-    <t>Take 001</t>
-  </si>
-  <si>
-    <t>EXPLOMED</t>
-  </si>
-  <si>
-    <t>可产出枪兵和近战兵</t>
-  </si>
-  <si>
-    <t>民房</t>
-  </si>
-  <si>
-    <t>建筑/民房</t>
-  </si>
-  <si>
-    <t>地堡</t>
-  </si>
-  <si>
-    <t>建筑/地堡</t>
-  </si>
-  <si>
-    <t>地堡872面</t>
-  </si>
-  <si>
-    <t>高HP，可派遣步兵进入地堡</t>
-  </si>
-  <si>
-    <t>炮台</t>
-  </si>
-  <si>
-    <t>建筑/炮台</t>
-  </si>
-  <si>
-    <t>p_jiqiangbao_d_01</t>
-  </si>
-  <si>
-    <t>show</t>
-  </si>
-  <si>
-    <t>音效/explo1</t>
-  </si>
-  <si>
-    <t>克制除了坦克以外的一切单位</t>
-  </si>
-  <si>
-    <t>虫巢</t>
-  </si>
-  <si>
-    <t>建筑/虫巢</t>
-  </si>
-  <si>
-    <t>音效/zhaWht00</t>
-  </si>
-  <si>
-    <t>hatchery_skin</t>
-  </si>
-  <si>
-    <t>音效/ZBldgDth</t>
-  </si>
-  <si>
-    <t>可产出幼虫</t>
-  </si>
-  <si>
-    <t>机场</t>
-  </si>
-  <si>
-    <t>建筑/机场</t>
-  </si>
-  <si>
-    <t>airport_500_1mesh</t>
-  </si>
-  <si>
-    <t>可产出飞机</t>
-  </si>
-  <si>
-    <t>重车厂</t>
-  </si>
-  <si>
-    <t>建筑/重车厂</t>
-  </si>
-  <si>
-    <t>风扇飞</t>
-  </si>
-  <si>
-    <t>重车厂Idle</t>
-  </si>
-  <si>
-    <t>可产出三色坦克</t>
-  </si>
-  <si>
-    <t>虫营</t>
-  </si>
-  <si>
-    <t>建筑/虫营</t>
-  </si>
-  <si>
-    <t>音效/zspWht00</t>
-  </si>
-  <si>
-    <t>近战虫和枪虫的前置建筑，只需1个就够了</t>
-  </si>
-  <si>
-    <t>飞塔</t>
-  </si>
-  <si>
-    <t>建筑/飞塔</t>
-  </si>
-  <si>
-    <t>音效/zscWht00</t>
-  </si>
-  <si>
-    <t>飞虫的前置建筑，只需1个就够了</t>
-  </si>
-  <si>
-    <t>拟态源</t>
-  </si>
-  <si>
-    <t>建筑/拟态源</t>
-  </si>
-  <si>
-    <t>绿色坦克的前置建筑，只需1个就够了</t>
-  </si>
-  <si>
-    <t>太岁</t>
-  </si>
-  <si>
-    <t>建筑/太岁</t>
-  </si>
-  <si>
-    <t>可扩张苔蔓(wàn)，扩张完成后可分裂另一个太岁</t>
-  </si>
-  <si>
-    <t>枪虫怪</t>
-  </si>
-  <si>
-    <t>近战虫怪</t>
-  </si>
-  <si>
-    <t>工怪</t>
   </si>
   <si>
     <t>枪兵怪</t>
@@ -4136,7 +4139,7 @@
         <v>59</v>
       </c>
       <c r="E37" s="11" t="s">
-        <v>60</v>
+        <v>177</v>
       </c>
       <c r="F37" s="11" t="s">
         <v>61</v>
@@ -4180,13 +4183,13 @@
         <v>404</v>
       </c>
       <c r="B38" s="24" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C38" s="11">
         <v>1</v>
       </c>
       <c r="D38" s="11" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="E38" s="11" t="s">
         <v>41</v>
@@ -4230,7 +4233,7 @@
         <v>405</v>
       </c>
       <c r="B39" s="24" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C39">
         <v>1</v>
@@ -4289,7 +4292,7 @@
         <v>406</v>
       </c>
       <c r="B40" s="24" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C40" s="11">
         <v>1</v>
@@ -4342,7 +4345,7 @@
         <v>407</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C41">
         <v>2</v>
@@ -4398,7 +4401,7 @@
         <v>408</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C42">
         <v>2</v>
@@ -4454,7 +4457,7 @@
         <v>409</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C43">
         <v>2</v>
@@ -4510,7 +4513,7 @@
         <v>410</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C44">
         <v>2</v>
@@ -4587,22 +4590,22 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
     </row>
     <row r="2" s="1" customFormat="1" spans="1:5">
@@ -4610,16 +4613,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
     </row>
     <row r="3" s="1" customFormat="1" spans="1:5">
@@ -4627,16 +4630,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="C3" t="s">
+        <v>295</v>
+      </c>
+      <c r="D3" t="s">
+        <v>296</v>
+      </c>
+      <c r="E3" s="4" t="s">
         <v>297</v>
-      </c>
-      <c r="C3" t="s">
-        <v>294</v>
-      </c>
-      <c r="D3" t="s">
-        <v>295</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>296</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -4644,16 +4647,16 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C4" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D4" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -4661,16 +4664,16 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
+        <v>303</v>
+      </c>
+      <c r="C5" t="s">
+        <v>300</v>
+      </c>
+      <c r="D5" t="s">
+        <v>301</v>
+      </c>
+      <c r="E5" s="4" t="s">
         <v>302</v>
-      </c>
-      <c r="C5" t="s">
-        <v>299</v>
-      </c>
-      <c r="D5" t="s">
-        <v>300</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>301</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -4678,16 +4681,16 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C6" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D6" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="E6" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -4695,16 +4698,16 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
+        <v>306</v>
+      </c>
+      <c r="C7" t="s">
+        <v>295</v>
+      </c>
+      <c r="D7" t="s">
+        <v>296</v>
+      </c>
+      <c r="E7" t="s">
         <v>305</v>
-      </c>
-      <c r="C7" t="s">
-        <v>294</v>
-      </c>
-      <c r="D7" t="s">
-        <v>295</v>
-      </c>
-      <c r="E7" t="s">
-        <v>304</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -4712,16 +4715,16 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C8" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="D8" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E8" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -4729,16 +4732,16 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
+        <v>311</v>
+      </c>
+      <c r="C9" t="s">
+        <v>308</v>
+      </c>
+      <c r="D9" t="s">
+        <v>309</v>
+      </c>
+      <c r="E9" t="s">
         <v>310</v>
-      </c>
-      <c r="C9" t="s">
-        <v>307</v>
-      </c>
-      <c r="D9" t="s">
-        <v>308</v>
-      </c>
-      <c r="E9" t="s">
-        <v>309</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -4746,16 +4749,16 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D10" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E10" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -4763,16 +4766,16 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C11" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D11" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E11" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
     </row>
     <row r="12" ht="14.25" spans="1:7">
@@ -4780,22 +4783,22 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C12" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="D12" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -4803,16 +4806,16 @@
         <v>101</v>
       </c>
       <c r="B13" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C13" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D13" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="14" ht="14.25" spans="1:7">
@@ -4820,22 +4823,22 @@
         <v>102</v>
       </c>
       <c r="B14" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C14" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D14" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -4843,16 +4846,16 @@
         <v>201</v>
       </c>
       <c r="B15" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C15" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D15" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="E15" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
     </row>
     <row r="16" ht="14.25" spans="1:7">
@@ -4860,22 +4863,22 @@
         <v>202</v>
       </c>
       <c r="B16" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="C16" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="D16" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
   </sheetData>
@@ -4905,10 +4908,10 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C1" s="1"/>
     </row>
@@ -4917,7 +4920,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -4925,7 +4928,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
     </row>
   </sheetData>
@@ -4950,22 +4953,22 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="2" s="1" customFormat="1" spans="1:7">
@@ -5140,7 +5143,7 @@
         <v>6</v>
       </c>
       <c r="D9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E9">
         <v>15</v>
@@ -5163,7 +5166,7 @@
         <v>3</v>
       </c>
       <c r="D10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E10">
         <v>12</v>
@@ -5637,22 +5640,22 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C1" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="G1" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -5729,7 +5732,7 @@
         <v>4</v>
       </c>
       <c r="D5" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -5975,25 +5978,25 @@
         <v>0</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E1" s="12" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="H1" s="12" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -6004,7 +6007,7 @@
         <v>33</v>
       </c>
       <c r="C2" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D2">
         <v>0</v>
@@ -6019,7 +6022,7 @@
         <v>35</v>
       </c>
       <c r="H2" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -6030,10 +6033,10 @@
         <v>39</v>
       </c>
       <c r="C3" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D3" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -6045,7 +6048,7 @@
         <v>41</v>
       </c>
       <c r="H3" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -6056,7 +6059,7 @@
         <v>46</v>
       </c>
       <c r="C4" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -6071,7 +6074,7 @@
         <v>41</v>
       </c>
       <c r="H4" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -6082,10 +6085,10 @@
         <v>52</v>
       </c>
       <c r="C5" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D5" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -6097,7 +6100,7 @@
         <v>54</v>
       </c>
       <c r="H5" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -6108,10 +6111,10 @@
         <v>58</v>
       </c>
       <c r="C6" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -6120,10 +6123,10 @@
         <v>0</v>
       </c>
       <c r="G6" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="H6" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="7" ht="14.25" spans="1:8">
@@ -6149,7 +6152,7 @@
         <v>67</v>
       </c>
       <c r="H7" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -6160,10 +6163,10 @@
         <v>72</v>
       </c>
       <c r="C8" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D8" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E8">
         <v>0</v>
@@ -6172,10 +6175,10 @@
         <v>0.7</v>
       </c>
       <c r="G8" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="H8" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -6186,10 +6189,10 @@
         <v>77</v>
       </c>
       <c r="C9" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D9" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E9">
         <v>0</v>
@@ -6198,10 +6201,10 @@
         <v>0</v>
       </c>
       <c r="G9" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="H9" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -6215,7 +6218,7 @@
         <v>84</v>
       </c>
       <c r="D10" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E10">
         <v>0</v>
@@ -6238,10 +6241,10 @@
         <v>90</v>
       </c>
       <c r="C11" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D11" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E11">
         <v>0</v>
@@ -6250,10 +6253,10 @@
         <v>0</v>
       </c>
       <c r="G11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="H11" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="12" customFormat="1" spans="1:6">
@@ -6278,7 +6281,7 @@
         <v>97</v>
       </c>
       <c r="C13" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D13" t="s">
         <v>100</v>
@@ -6290,10 +6293,10 @@
         <v>0</v>
       </c>
       <c r="G13" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="H13" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="14" customFormat="1" spans="1:8">
@@ -6304,7 +6307,7 @@
         <v>104</v>
       </c>
       <c r="C14" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="D14" t="s">
         <v>100</v>
@@ -6316,10 +6319,10 @@
         <v>0</v>
       </c>
       <c r="G14" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="H14" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="15" customFormat="1" spans="1:8">
@@ -6330,7 +6333,7 @@
         <v>110</v>
       </c>
       <c r="C15" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D15">
         <v>1</v>
@@ -6342,10 +6345,10 @@
         <v>0</v>
       </c>
       <c r="G15" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="H15" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="16" customFormat="1" spans="1:8">
@@ -6356,10 +6359,10 @@
         <v>116</v>
       </c>
       <c r="C16" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D16" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E16">
         <v>0</v>
@@ -6371,7 +6374,7 @@
         <v>41</v>
       </c>
       <c r="H16" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -6382,10 +6385,10 @@
         <v>174</v>
       </c>
       <c r="C17" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D17" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E17">
         <v>0</v>
@@ -6402,10 +6405,10 @@
         <v>175</v>
       </c>
       <c r="C18" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D18" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E18">
         <v>0</v>
@@ -6422,10 +6425,10 @@
         <v>176</v>
       </c>
       <c r="C19" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D19" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E19">
         <v>0</v>
@@ -6439,13 +6442,13 @@
         <v>404</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C20" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D20" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E20">
         <v>0</v>
@@ -6457,7 +6460,7 @@
         <v>41</v>
       </c>
       <c r="H20" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -6465,10 +6468,10 @@
         <v>405</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C21" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D21">
         <v>1</v>
@@ -6483,7 +6486,7 @@
         <v>41</v>
       </c>
       <c r="H21" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -6491,10 +6494,10 @@
         <v>406</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C22" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D22">
         <v>0</v>
@@ -6509,7 +6512,7 @@
         <v>35</v>
       </c>
       <c r="H22" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -6517,13 +6520,13 @@
         <v>407</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C23" t="s">
         <v>84</v>
       </c>
       <c r="D23" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E23">
         <v>0</v>
@@ -6543,10 +6546,10 @@
         <v>408</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C24" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="D24" t="s">
         <v>100</v>
@@ -6558,10 +6561,10 @@
         <v>0</v>
       </c>
       <c r="G24" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="H24" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -6569,13 +6572,13 @@
         <v>409</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C25" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D25" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E25">
         <v>0</v>
@@ -6584,10 +6587,10 @@
         <v>0</v>
       </c>
       <c r="G25" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="H25" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -6595,10 +6598,10 @@
         <v>410</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C26" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D26" t="s">
         <v>100</v>
@@ -6610,10 +6613,10 @@
         <v>0</v>
       </c>
       <c r="G26" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="H26" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
   </sheetData>
@@ -6662,64 +6665,64 @@
         <v>0</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="E1" s="12" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="H1" s="12" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="I1" s="12" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="J1" s="9" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="K1" s="12" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="L1" s="12" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="M1" s="12" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="N1" s="12" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="O1" s="12" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="P1" s="12" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="Q1" s="12" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="R1" s="12" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="S1" s="12" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="T1" s="12" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="U1" s="12" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="2" spans="1:21">
@@ -6763,7 +6766,7 @@
         <v>500</v>
       </c>
       <c r="Q2" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="R2">
         <v>500</v>
@@ -6804,7 +6807,7 @@
         <v>0</v>
       </c>
       <c r="J3" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="K3">
         <v>1</v>
@@ -6816,7 +6819,7 @@
         <v>0</v>
       </c>
       <c r="N3" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="O3">
         <v>2.5</v>
@@ -6825,7 +6828,7 @@
         <v>900</v>
       </c>
       <c r="Q3" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="R3">
         <v>100</v>
@@ -6881,7 +6884,7 @@
         <v>1300</v>
       </c>
       <c r="Q4" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="R4">
         <v>500</v>
@@ -6925,7 +6928,7 @@
         <v>5000</v>
       </c>
       <c r="J5" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="K5">
         <v>1</v>
@@ -6937,13 +6940,13 @@
         <v>0</v>
       </c>
       <c r="N5" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="P5">
         <v>300</v>
       </c>
       <c r="Q5" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="R5">
         <v>100</v>
@@ -6984,7 +6987,7 @@
         <v>0</v>
       </c>
       <c r="J6" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="K6">
         <v>1</v>
@@ -6999,7 +7002,7 @@
         <v>500</v>
       </c>
       <c r="Q6" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="R6">
         <v>300</v>
@@ -7052,7 +7055,7 @@
         <v>2</v>
       </c>
       <c r="N7" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="O7">
         <v>5</v>
@@ -7061,7 +7064,7 @@
         <v>800</v>
       </c>
       <c r="Q7" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="R7">
         <v>100</v>
@@ -7102,7 +7105,7 @@
         <v>0</v>
       </c>
       <c r="J8" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="K8">
         <v>1</v>
@@ -7114,7 +7117,7 @@
         <v>0</v>
       </c>
       <c r="N8" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="O8">
         <v>1</v>
@@ -7123,7 +7126,7 @@
         <v>300</v>
       </c>
       <c r="Q8" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="R8">
         <v>600</v>
@@ -7164,7 +7167,7 @@
         <v>0</v>
       </c>
       <c r="J9" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="K9">
         <v>1</v>
@@ -7179,7 +7182,7 @@
         <v>570</v>
       </c>
       <c r="Q9" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="R9">
         <v>1030</v>
@@ -7220,7 +7223,7 @@
         <v>0</v>
       </c>
       <c r="J10" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="K10">
         <v>1</v>
@@ -7235,7 +7238,7 @@
         <v>600</v>
       </c>
       <c r="Q10" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="R10">
         <v>200</v>
@@ -7279,7 +7282,7 @@
         <v>0</v>
       </c>
       <c r="J11" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="K11">
         <v>1</v>
@@ -7294,7 +7297,7 @@
         <v>500</v>
       </c>
       <c r="Q11" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="R11">
         <v>900</v>
@@ -7347,7 +7350,7 @@
         <v>0</v>
       </c>
       <c r="Q12" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="R12">
         <v>0</v>
@@ -7447,7 +7450,7 @@
         <v>0</v>
       </c>
       <c r="N14" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="O14">
         <v>5</v>
@@ -7456,7 +7459,7 @@
         <v>600</v>
       </c>
       <c r="Q14" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="R14">
         <v>300</v>
@@ -7512,7 +7515,7 @@
         <v>1000</v>
       </c>
       <c r="Q15" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="R15">
         <v>100</v>
@@ -7553,7 +7556,7 @@
         <v>1000</v>
       </c>
       <c r="J16" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="K16">
         <v>1</v>
@@ -7565,7 +7568,7 @@
         <v>0</v>
       </c>
       <c r="N16" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="O16">
         <v>2.5</v>
@@ -7574,7 +7577,7 @@
         <v>530</v>
       </c>
       <c r="Q16" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="R16">
         <v>100</v>
@@ -7863,7 +7866,7 @@
         <v>0</v>
       </c>
       <c r="N21" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="O21">
         <v>4</v>
@@ -7872,7 +7875,7 @@
         <v>400</v>
       </c>
       <c r="Q21" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="R21">
         <v>400</v>
@@ -8326,7 +8329,7 @@
         <v>0</v>
       </c>
       <c r="J29" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="K29">
         <v>1</v>
@@ -8338,7 +8341,7 @@
         <v>0</v>
       </c>
       <c r="N29" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="O29">
         <v>1</v>
@@ -8347,7 +8350,7 @@
         <v>300</v>
       </c>
       <c r="Q29" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="R29">
         <v>600</v>
@@ -8388,7 +8391,7 @@
         <v>0</v>
       </c>
       <c r="J30" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="K30">
         <v>1</v>
@@ -8403,7 +8406,7 @@
         <v>570</v>
       </c>
       <c r="Q30" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="R30">
         <v>1030</v>
@@ -8444,7 +8447,7 @@
         <v>0</v>
       </c>
       <c r="J31" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="K31">
         <v>1</v>
@@ -8459,7 +8462,7 @@
         <v>600</v>
       </c>
       <c r="Q31" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="R31">
         <v>300</v>
@@ -8479,7 +8482,7 @@
         <v>404</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C32">
         <v>20</v>
@@ -8500,7 +8503,7 @@
         <v>0</v>
       </c>
       <c r="J32" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="K32">
         <v>1</v>
@@ -8512,7 +8515,7 @@
         <v>0</v>
       </c>
       <c r="N32" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="O32">
         <v>4</v>
@@ -8521,7 +8524,7 @@
         <v>900</v>
       </c>
       <c r="Q32" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="R32">
         <v>100</v>
@@ -8541,7 +8544,7 @@
         <v>405</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C33">
         <v>15</v>
@@ -8577,7 +8580,7 @@
         <v>1300</v>
       </c>
       <c r="Q33" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="R33">
         <v>500</v>
@@ -8597,7 +8600,7 @@
         <v>406</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C34">
         <v>12</v>
@@ -8633,7 +8636,7 @@
         <v>500</v>
       </c>
       <c r="Q34" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="R34">
         <v>500</v>
@@ -8653,7 +8656,7 @@
         <v>407</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C35">
         <v>0</v>
@@ -8674,7 +8677,7 @@
         <v>0</v>
       </c>
       <c r="J35" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="K35">
         <v>1</v>
@@ -8689,7 +8692,7 @@
         <v>600</v>
       </c>
       <c r="Q35" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="R35">
         <v>200</v>
@@ -8709,7 +8712,7 @@
         <v>408</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C36">
         <v>30</v>
@@ -8739,7 +8742,7 @@
         <v>0</v>
       </c>
       <c r="N36" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="O36">
         <v>5</v>
@@ -8748,7 +8751,7 @@
         <v>600</v>
       </c>
       <c r="Q36" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="R36">
         <v>300</v>
@@ -8768,7 +8771,7 @@
         <v>409</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C37">
         <v>35</v>
@@ -8792,7 +8795,7 @@
         <v>0</v>
       </c>
       <c r="J37" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="K37">
         <v>1</v>
@@ -8807,7 +8810,7 @@
         <v>500</v>
       </c>
       <c r="Q37" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="R37">
         <v>900</v>
@@ -8827,7 +8830,7 @@
         <v>410</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C38">
         <v>0</v>
@@ -8889,10 +8892,10 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C1" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -8944,7 +8947,7 @@
         <v>401</v>
       </c>
       <c r="B6" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C6">
         <v>15</v>
@@ -8955,7 +8958,7 @@
         <v>402</v>
       </c>
       <c r="B7" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C7">
         <v>12</v>
@@ -8977,7 +8980,7 @@
         <v>404</v>
       </c>
       <c r="B9" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C9">
         <v>15</v>
@@ -8988,7 +8991,7 @@
         <v>405</v>
       </c>
       <c r="B10" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C10">
         <v>20</v>
@@ -8999,7 +9002,7 @@
         <v>406</v>
       </c>
       <c r="B11" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C11">
         <v>25</v>
@@ -9010,7 +9013,7 @@
         <v>407</v>
       </c>
       <c r="B12" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C12">
         <v>10</v>
@@ -9021,7 +9024,7 @@
         <v>408</v>
       </c>
       <c r="B13" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C13">
         <v>20</v>
@@ -9032,7 +9035,7 @@
         <v>409</v>
       </c>
       <c r="B14" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C14">
         <v>30</v>
@@ -9043,7 +9046,7 @@
         <v>410</v>
       </c>
       <c r="B15" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C15">
         <v>45</v>
@@ -9069,25 +9072,25 @@
         <v>0</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="H1" s="9" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -9098,7 +9101,7 @@
         <v>39</v>
       </c>
       <c r="C2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -9124,7 +9127,7 @@
         <v>46</v>
       </c>
       <c r="C3" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D3">
         <v>2</v>
@@ -9150,7 +9153,7 @@
         <v>52</v>
       </c>
       <c r="C4" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D4">
         <v>4</v>
@@ -9176,7 +9179,7 @@
         <v>65</v>
       </c>
       <c r="C5" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D5">
         <v>5</v>
@@ -9202,7 +9205,7 @@
         <v>72</v>
       </c>
       <c r="C6" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D6">
         <v>2</v>
@@ -9228,7 +9231,7 @@
         <v>77</v>
       </c>
       <c r="C7" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -9254,7 +9257,7 @@
         <v>90</v>
       </c>
       <c r="C8" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D8">
         <v>5</v>
@@ -9280,7 +9283,7 @@
         <v>104</v>
       </c>
       <c r="C9" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D9">
         <v>4</v>
@@ -9318,13 +9321,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -9372,19 +9375,19 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C1" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="D1" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="E1" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -9392,7 +9395,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C2">
         <v>4</v>
@@ -9409,7 +9412,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C3">
         <v>3</v>
@@ -9426,7 +9429,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C4">
         <v>3</v>
@@ -9443,7 +9446,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C5">
         <v>3</v>
@@ -9460,7 +9463,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C6">
         <v>8</v>
@@ -9477,7 +9480,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C7">
         <v>8</v>
@@ -9494,7 +9497,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C8">
         <v>8</v>

</xml_diff>